<commit_message>
Save library recording Session 11/10/2026, 14:42:14 - 5c86e5ce-1c83-4894-8aa4-b77e1d2b737b - 2026-10-11T03:43:45.132102Z
</commit_message>
<xml_diff>
--- a/library/projects/1c7a86a9-9525-4bd4-b5f0-df360a7b49f1/recordings/5c86e5ce-1c83-4894-8aa4-b77e1d2b737b/resources/azure-devops.xlsx
+++ b/library/projects/1c7a86a9-9525-4bd4-b5f0-df360a7b49f1/recordings/5c86e5ce-1c83-4894-8aa4-b77e1d2b737b/resources/azure-devops.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -445,6 +445,122 @@
       <c r="F1" t="inlineStr">
         <is>
           <t>Screenshot</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Session 11/10/2026, 14:42:14</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Open https://hfm-wholesale-app-dev.ashysand-8cabb4df.australiaeast.azurecontainerapps.io/daily-orders?storeNo=426&amp;date=2026-10-08</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>https://hfm-wholesale-app-dev.ashysand-8cabb4df.australiaeast.azurecontainerapps.io/daily-orders?storeNo=426&amp;date=2026-10-08</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Session 11/10/2026, 14:42:14</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Click 123,322</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>{"primary": "div:nth-of-type(1) &gt; div:nth-of-type(2) &gt; div:nth-of-type(1) &gt; form:nth-of-type(1) &gt; label:nth-of-type(1) &gt; input:nth-of-type(1)", "x": 123, "y": 322, "text": "", "tag": "input"}</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>step-002.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Session 11/10/2026, 14:42:14</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Type: Ratta</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Ratta</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>{"primary": "div:nth-of-type(1) &gt; div:nth-of-type(2) &gt; div:nth-of-type(1) &gt; form:nth-of-type(1) &gt; label:nth-of-type(1) &gt; input:nth-of-type(1)"}</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>step-003.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Session 11/10/2026, 14:42:14</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Click 115,416</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>{"primary": "div:nth-of-type(1) &gt; div:nth-of-type(2) &gt; div:nth-of-type(1) &gt; form:nth-of-type(1) &gt; label:nth-of-type(2) &gt; input:nth-of-type(1)", "x": 115, "y": 416, "text": "", "tag": "input"}</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>step-004.png</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Save library recording Session 11/10/2026, 14:42:14 - 5c86e5ce-1c83-4894-8aa4-b77e1d2b737b - 2026-10-11T13:04:51.714711Z
</commit_message>
<xml_diff>
--- a/library/projects/1c7a86a9-9525-4bd4-b5f0-df360a7b49f1/recordings/5c86e5ce-1c83-4894-8aa4-b77e1d2b737b/resources/azure-devops.xlsx
+++ b/library/projects/1c7a86a9-9525-4bd4-b5f0-df360a7b49f1/recordings/5c86e5ce-1c83-4894-8aa4-b77e1d2b737b/resources/azure-devops.xlsx
@@ -495,7 +495,7 @@
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>{"primary": "div:nth-of-type(1) &gt; div:nth-of-type(2) &gt; div:nth-of-type(1) &gt; form:nth-of-type(1) &gt; label:nth-of-type(1) &gt; input:nth-of-type(1)", "x": 123, "y": 322, "text": "", "tag": "input"}</t>
+          <t>{"primary": "div:nth-of-type(1) &gt; div:nth-of-type(2) &gt; div:nth-of-type(1) &gt; form:nth-of-type(1) &gt; label:nth-of-type(1) &gt; input:nth-of-type(1)", "tag": "input", "text": "", "x": 123, "y": 322}</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -517,12 +517,12 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Type: Ratta</t>
+          <t>Type: Sa</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Ratta</t>
+          <t>Sa</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -555,7 +555,7 @@
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>{"primary": "div:nth-of-type(1) &gt; div:nth-of-type(2) &gt; div:nth-of-type(1) &gt; form:nth-of-type(1) &gt; label:nth-of-type(2) &gt; input:nth-of-type(1)", "x": 115, "y": 416, "text": "", "tag": "input"}</t>
+          <t>{"primary": "div:nth-of-type(1) &gt; div:nth-of-type(2) &gt; div:nth-of-type(1) &gt; form:nth-of-type(1) &gt; label:nth-of-type(2) &gt; input:nth-of-type(1)", "tag": "input", "text": "", "x": 115, "y": 416}</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">

</xml_diff>